<commit_message>
DEJO UNA SOLA COLUMNA PARA 1-2-3
</commit_message>
<xml_diff>
--- a/Tabla de transiciones.xlsx
+++ b/Tabla de transiciones.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\javier\unahur\Parseo\prototipo-de-lenguaje\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\UNAHUR - PARSEO\TP\prototipo-de-lenguaje\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA5430AD-51BE-4D27-8B75-E43B51F58A2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{671EE0FE-EA9D-4299-A6FC-B98C3CAAB297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="-75" windowWidth="24240" windowHeight="13140" xr2:uid="{5429F7BC-090D-44AD-AC20-D5F60C384123}"/>
+    <workbookView xWindow="5985" yWindow="3465" windowWidth="21600" windowHeight="11505" xr2:uid="{5429F7BC-090D-44AD-AC20-D5F60C384123}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -31,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="29">
   <si>
     <t>Q</t>
   </si>
@@ -122,13 +125,7 @@
     <t>otras(a-z)</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
+    <t>1 - 2 - 3</t>
   </si>
 </sst>
 </file>
@@ -182,13 +179,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="23">
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -272,31 +263,29 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1AAA77F-CD3C-4BB2-9327-99EFB459C579}" name="Tabla1" displayName="Tabla1" ref="A2:W35" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
-  <tableColumns count="23">
-    <tableColumn id="1" xr3:uid="{DCEA3D7F-93B1-4A0A-9B4B-F6F76FD1C464}" name="Q" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{1BCD12BF-0F6B-4309-9877-3526B3926E76}" name="+" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{F235F50D-9E4E-4FE5-A90F-57B89FEEEA8C}" name="=" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{3273E231-2914-407C-A580-83C35015E7EC}" name="b" dataDxfId="19"/>
-    <tableColumn id="16" xr3:uid="{7A620641-516D-4500-A316-7BF5975EEA91}" name="d" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{99C2B348-4DD3-4433-BBEE-EE0E4DC09ADF}" name="e" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{A681EC8B-4183-4F10-9A4E-C7C90560DC22}" name="f" dataDxfId="16"/>
-    <tableColumn id="17" xr3:uid="{2EC1F855-441D-489A-B440-DA93EBEFF149}" name="g" dataDxfId="15"/>
-    <tableColumn id="15" xr3:uid="{B3EE192B-1C77-4E83-8336-6CA44D2F82F1}" name="i" dataDxfId="14"/>
-    <tableColumn id="21" xr3:uid="{C53971FA-CC6F-418C-806D-B10ABB739F56}" name="l" dataDxfId="13"/>
-    <tableColumn id="22" xr3:uid="{5BDC76FC-4A24-41A6-B059-3D5CC7975BAD}" name="n" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{69A340D6-DEDF-4E8C-B338-58DB8E0498E7}" name="p" dataDxfId="11"/>
-    <tableColumn id="18" xr3:uid="{01AA33C5-3B41-4650-A51E-839DD2D96FBA}" name="r" dataDxfId="10"/>
-    <tableColumn id="19" xr3:uid="{A6776B4A-7E79-4374-8593-C1D71D5351B0}" name="s" dataDxfId="9"/>
-    <tableColumn id="20" xr3:uid="{8A5A32F0-5A6F-4982-9E67-31C9C05CBE7D}" name="t" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{43596D7C-A795-4530-8C5B-9E8E98E09890}" name="otras(a-z)" dataDxfId="7"/>
-    <tableColumn id="11" xr3:uid="{D6DF204D-7DA8-40FD-9A25-041C2D166B52}" name="(" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{E40B259A-D566-4A6B-AF8A-418FA02CDDC9}" name=")" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{42279991-C553-43DA-87B5-C38C90202F8B}" name="1" dataDxfId="4"/>
-    <tableColumn id="23" xr3:uid="{A4986637-C124-4458-BCF6-300BAA98EC02}" name="2" dataDxfId="1"/>
-    <tableColumn id="24" xr3:uid="{A0E13203-721A-4D55-9C6C-F2003E920F8E}" name="3" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{CB21011E-A48F-487A-A96A-51D2C6084C30}" name="Token" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{EEAC61DA-BA95-4111-A22D-DFF27BF4A58C}" name="Retroceso" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1AAA77F-CD3C-4BB2-9327-99EFB459C579}" name="Tabla1" displayName="Tabla1" ref="A2:U35" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <tableColumns count="21">
+    <tableColumn id="1" xr3:uid="{DCEA3D7F-93B1-4A0A-9B4B-F6F76FD1C464}" name="Q" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{1BCD12BF-0F6B-4309-9877-3526B3926E76}" name="+" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{F235F50D-9E4E-4FE5-A90F-57B89FEEEA8C}" name="=" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{3273E231-2914-407C-A580-83C35015E7EC}" name="b" dataDxfId="17"/>
+    <tableColumn id="16" xr3:uid="{7A620641-516D-4500-A316-7BF5975EEA91}" name="d" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{99C2B348-4DD3-4433-BBEE-EE0E4DC09ADF}" name="e" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{A681EC8B-4183-4F10-9A4E-C7C90560DC22}" name="f" dataDxfId="14"/>
+    <tableColumn id="17" xr3:uid="{2EC1F855-441D-489A-B440-DA93EBEFF149}" name="g" dataDxfId="13"/>
+    <tableColumn id="15" xr3:uid="{B3EE192B-1C77-4E83-8336-6CA44D2F82F1}" name="i" dataDxfId="12"/>
+    <tableColumn id="21" xr3:uid="{C53971FA-CC6F-418C-806D-B10ABB739F56}" name="l" dataDxfId="11"/>
+    <tableColumn id="22" xr3:uid="{5BDC76FC-4A24-41A6-B059-3D5CC7975BAD}" name="n" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{69A340D6-DEDF-4E8C-B338-58DB8E0498E7}" name="p" dataDxfId="9"/>
+    <tableColumn id="18" xr3:uid="{01AA33C5-3B41-4650-A51E-839DD2D96FBA}" name="r" dataDxfId="8"/>
+    <tableColumn id="19" xr3:uid="{A6776B4A-7E79-4374-8593-C1D71D5351B0}" name="s" dataDxfId="7"/>
+    <tableColumn id="20" xr3:uid="{8A5A32F0-5A6F-4982-9E67-31C9C05CBE7D}" name="t" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{43596D7C-A795-4530-8C5B-9E8E98E09890}" name="otras(a-z)" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{D6DF204D-7DA8-40FD-9A25-041C2D166B52}" name="(" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{E40B259A-D566-4A6B-AF8A-418FA02CDDC9}" name=")" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{42279991-C553-43DA-87B5-C38C90202F8B}" name="1 - 2 - 3" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{CB21011E-A48F-487A-A96A-51D2C6084C30}" name="Token" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{EEAC61DA-BA95-4111-A22D-DFF27BF4A58C}" name="Retroceso" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -619,14 +608,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1F50169-9F27-43B7-B1FB-1286865D0027}">
-  <dimension ref="A2:W35"/>
+  <dimension ref="A2:U35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="21" width="11.42578125" style="1"/>
-    <col min="22" max="22" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="19" width="11.42578125" style="1"/>
+    <col min="20" max="20" width="21.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -684,20 +673,14 @@
       <c r="S2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="T2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="V2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="U2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>0</v>
       </c>
@@ -755,20 +738,14 @@
       <c r="S3" s="1">
         <v>17</v>
       </c>
-      <c r="T3" s="1">
-        <v>17</v>
-      </c>
-      <c r="U3" s="1">
-        <v>17</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W3" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -827,19 +804,13 @@
         <v>1</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="V4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="1">
+      <c r="U4" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>2</v>
       </c>
@@ -897,20 +868,14 @@
       <c r="S5" s="1">
         <v>33</v>
       </c>
-      <c r="T5" s="1">
-        <v>33</v>
-      </c>
-      <c r="U5" s="1">
-        <v>33</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W5" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>3</v>
       </c>
@@ -968,20 +933,14 @@
       <c r="S6" s="1">
         <v>18</v>
       </c>
-      <c r="T6" s="1">
-        <v>18</v>
-      </c>
-      <c r="U6" s="1">
-        <v>18</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W6" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -1040,19 +999,13 @@
         <v>1</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="V7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="W7" s="1">
+      <c r="U7" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -1110,20 +1063,14 @@
       <c r="S8" s="1">
         <v>7</v>
       </c>
-      <c r="T8" s="1">
-        <v>8</v>
-      </c>
-      <c r="U8" s="1">
-        <v>9</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W8" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U8" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -1182,19 +1129,13 @@
         <v>1</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W9" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="U9" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -1252,20 +1193,14 @@
       <c r="S10" s="1">
         <v>18</v>
       </c>
-      <c r="T10" s="1">
-        <v>18</v>
-      </c>
-      <c r="U10" s="1">
-        <v>18</v>
-      </c>
-      <c r="V10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W10" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U10" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -1323,20 +1258,14 @@
       <c r="S11" s="1">
         <v>21</v>
       </c>
-      <c r="T11" s="1">
-        <v>21</v>
-      </c>
-      <c r="U11" s="1">
-        <v>21</v>
-      </c>
-      <c r="V11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W11" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U11" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -1394,20 +1323,14 @@
       <c r="S12" s="1">
         <v>21</v>
       </c>
-      <c r="T12" s="1">
-        <v>21</v>
-      </c>
-      <c r="U12" s="1">
-        <v>21</v>
-      </c>
-      <c r="V12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W12" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U12" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -1465,20 +1388,14 @@
       <c r="S13" s="1">
         <v>21</v>
       </c>
-      <c r="T13" s="1">
-        <v>21</v>
-      </c>
-      <c r="U13" s="1">
-        <v>21</v>
-      </c>
-      <c r="V13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W13" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U13" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -1536,20 +1453,14 @@
       <c r="S14" s="1">
         <v>21</v>
       </c>
-      <c r="T14" s="1">
-        <v>21</v>
-      </c>
-      <c r="U14" s="1">
-        <v>21</v>
-      </c>
-      <c r="V14" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W14" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U14" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -1607,20 +1518,14 @@
       <c r="S15" s="1">
         <v>21</v>
       </c>
-      <c r="T15" s="1">
-        <v>21</v>
-      </c>
-      <c r="U15" s="1">
-        <v>21</v>
-      </c>
-      <c r="V15" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W15" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U15" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -1678,20 +1583,14 @@
       <c r="S16" s="1">
         <v>21</v>
       </c>
-      <c r="T16" s="1">
-        <v>21</v>
-      </c>
-      <c r="U16" s="1">
-        <v>21</v>
-      </c>
-      <c r="V16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W16" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U16" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -1749,20 +1648,14 @@
       <c r="S17" s="1">
         <v>21</v>
       </c>
-      <c r="T17" s="1">
-        <v>21</v>
-      </c>
-      <c r="U17" s="1">
-        <v>21</v>
-      </c>
-      <c r="V17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W17" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U17" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -1820,20 +1713,14 @@
       <c r="S18" s="1">
         <v>18</v>
       </c>
-      <c r="T18" s="1">
-        <v>18</v>
-      </c>
-      <c r="U18" s="1">
-        <v>18</v>
-      </c>
-      <c r="V18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W18" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U18" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -1892,19 +1779,13 @@
         <v>1</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="V19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="W19" s="1">
+      <c r="U19" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -1963,19 +1844,13 @@
         <v>1</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U20" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="V20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="W20" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="U20" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -2034,19 +1909,13 @@
         <v>1</v>
       </c>
       <c r="T21" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U21" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="V21" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="W21" s="1">
+      <c r="U21" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -2105,19 +1974,13 @@
         <v>1</v>
       </c>
       <c r="T22" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U22" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="V22" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="W22" s="1">
+      <c r="U22" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -2176,19 +2039,13 @@
         <v>1</v>
       </c>
       <c r="T23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="V23" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W23" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="U23" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -2246,20 +2103,14 @@
       <c r="S24" s="1">
         <v>18</v>
       </c>
-      <c r="T24" s="1">
-        <v>18</v>
-      </c>
-      <c r="U24" s="1">
-        <v>18</v>
-      </c>
-      <c r="V24" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W24" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U24" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -2317,20 +2168,14 @@
       <c r="S25" s="1">
         <v>33</v>
       </c>
-      <c r="T25" s="1">
-        <v>33</v>
-      </c>
-      <c r="U25" s="1">
-        <v>33</v>
-      </c>
-      <c r="V25" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W25" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T25" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U25" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -2388,20 +2233,14 @@
       <c r="S26" s="1">
         <v>33</v>
       </c>
-      <c r="T26" s="1">
-        <v>33</v>
-      </c>
-      <c r="U26" s="1">
-        <v>33</v>
-      </c>
-      <c r="V26" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W26" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U26" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -2459,20 +2298,14 @@
       <c r="S27" s="1">
         <v>33</v>
       </c>
-      <c r="T27" s="1">
-        <v>33</v>
-      </c>
-      <c r="U27" s="1">
-        <v>33</v>
-      </c>
-      <c r="V27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W27" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U27" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -2530,20 +2363,14 @@
       <c r="S28" s="1">
         <v>33</v>
       </c>
-      <c r="T28" s="1">
-        <v>33</v>
-      </c>
-      <c r="U28" s="1">
-        <v>33</v>
-      </c>
-      <c r="V28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W28" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T28" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U28" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -2601,20 +2428,14 @@
       <c r="S29" s="1">
         <v>18</v>
       </c>
-      <c r="T29" s="1">
-        <v>18</v>
-      </c>
-      <c r="U29" s="1">
-        <v>18</v>
-      </c>
-      <c r="V29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W29" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T29" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U29" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -2672,20 +2493,14 @@
       <c r="S30" s="1">
         <v>21</v>
       </c>
-      <c r="T30" s="1">
-        <v>21</v>
-      </c>
-      <c r="U30" s="1">
-        <v>21</v>
-      </c>
-      <c r="V30" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W30" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T30" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U30" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -2743,20 +2558,14 @@
       <c r="S31" s="1">
         <v>18</v>
       </c>
-      <c r="T31" s="1">
-        <v>18</v>
-      </c>
-      <c r="U31" s="1">
-        <v>18</v>
-      </c>
-      <c r="V31" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W31" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T31" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U31" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -2814,20 +2623,14 @@
       <c r="S32" s="1">
         <v>33</v>
       </c>
-      <c r="T32" s="1">
-        <v>33</v>
-      </c>
-      <c r="U32" s="1">
-        <v>33</v>
-      </c>
-      <c r="V32" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W32" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T32" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U32" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -2885,20 +2688,14 @@
       <c r="S33" s="1">
         <v>33</v>
       </c>
-      <c r="T33" s="1">
-        <v>33</v>
-      </c>
-      <c r="U33" s="1">
-        <v>33</v>
-      </c>
-      <c r="V33" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W33" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T33" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U33" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -2956,20 +2753,14 @@
       <c r="S34" s="1">
         <v>18</v>
       </c>
-      <c r="T34" s="1">
-        <v>18</v>
-      </c>
-      <c r="U34" s="1">
-        <v>18</v>
-      </c>
-      <c r="V34" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W34" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="T34" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U34" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -3028,15 +2819,9 @@
         <v>1</v>
       </c>
       <c r="T35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="V35" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W35" s="1">
+        <v>21</v>
+      </c>
+      <c r="U35" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
SE MODIFICAN TABLA TRNSICIONES Y GRAFICO POR NUEVOS TOKENS
</commit_message>
<xml_diff>
--- a/Tabla de transiciones.xlsx
+++ b/Tabla de transiciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\UNAHUR - PARSEO\TP\prototipo-de-lenguaje\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{671EE0FE-EA9D-4299-A6FC-B98C3CAAB297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B207F73-1148-4F8A-B43A-B737E4244587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5985" yWindow="3465" windowWidth="21600" windowHeight="11505" xr2:uid="{5429F7BC-090D-44AD-AC20-D5F60C384123}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{5429F7BC-090D-44AD-AC20-D5F60C384123}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="35">
   <si>
     <t>Q</t>
   </si>
@@ -101,9 +101,6 @@
     <t>s</t>
   </si>
   <si>
-    <t>PALABRA_RESERVADA</t>
-  </si>
-  <si>
     <t>ID</t>
   </si>
   <si>
@@ -126,6 +123,27 @@
   </si>
   <si>
     <t>1 - 2 - 3</t>
+  </si>
+  <si>
+    <t>END</t>
+  </si>
+  <si>
+    <t>ELSE</t>
+  </si>
+  <si>
+    <t>PRINT</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>IF</t>
+  </si>
+  <si>
+    <t>BEGIN</t>
+  </si>
+  <si>
+    <t>DEF</t>
   </si>
 </sst>
 </file>
@@ -263,7 +281,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1AAA77F-CD3C-4BB2-9327-99EFB459C579}" name="Tabla1" displayName="Tabla1" ref="A2:U35" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1AAA77F-CD3C-4BB2-9327-99EFB459C579}" name="Tabla1" displayName="Tabla1" ref="A2:U42" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{DCEA3D7F-93B1-4A0A-9B4B-F6F76FD1C464}" name="Q" dataDxfId="20"/>
     <tableColumn id="9" xr3:uid="{1BCD12BF-0F6B-4309-9877-3526B3926E76}" name="+" dataDxfId="19"/>
@@ -608,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1F50169-9F27-43B7-B1FB-1286865D0027}">
-  <dimension ref="A2:U35"/>
+  <dimension ref="A2:U42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="19" width="11.42578125" style="1"/>
@@ -626,10 +644,10 @@
         <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>7</v>
@@ -638,7 +656,7 @@
         <v>17</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>8</v>
@@ -650,10 +668,10 @@
         <v>16</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>19</v>
@@ -662,7 +680,7 @@
         <v>6</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q2" s="1" t="s">
         <v>9</v>
@@ -671,7 +689,7 @@
         <v>10</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>2</v>
@@ -880,10 +898,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="1">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="C6" s="1">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="D6" s="1">
         <v>6</v>
@@ -925,13 +943,13 @@
         <v>6</v>
       </c>
       <c r="Q6" s="1">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="R6" s="1">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="S6" s="1">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="T6" s="1" t="s">
         <v>1</v>
@@ -942,7 +960,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>1</v>
@@ -999,216 +1017,216 @@
         <v>1</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="U7" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>6</v>
-      </c>
-      <c r="B8" s="1">
-        <v>7</v>
-      </c>
-      <c r="C8" s="1">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1">
-        <v>6</v>
-      </c>
-      <c r="E8" s="1">
-        <v>6</v>
-      </c>
-      <c r="F8" s="1">
-        <v>6</v>
-      </c>
-      <c r="G8" s="1">
-        <v>6</v>
-      </c>
-      <c r="H8" s="1">
-        <v>6</v>
-      </c>
-      <c r="I8" s="1">
-        <v>6</v>
-      </c>
-      <c r="J8" s="1">
-        <v>6</v>
-      </c>
-      <c r="K8" s="1">
-        <v>6</v>
-      </c>
-      <c r="L8" s="1">
-        <v>6</v>
-      </c>
-      <c r="M8" s="1">
-        <v>6</v>
-      </c>
-      <c r="N8" s="1">
-        <v>6</v>
-      </c>
-      <c r="O8" s="1">
-        <v>6</v>
-      </c>
-      <c r="P8" s="1">
-        <v>6</v>
-      </c>
-      <c r="Q8" s="1">
-        <v>7</v>
-      </c>
-      <c r="R8" s="1">
-        <v>7</v>
-      </c>
-      <c r="S8" s="1">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="U8" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="S9" s="1" t="s">
-        <v>1</v>
+      <c r="C9" s="1">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1">
+        <v>6</v>
+      </c>
+      <c r="F9" s="1">
+        <v>6</v>
+      </c>
+      <c r="G9" s="1">
+        <v>6</v>
+      </c>
+      <c r="H9" s="1">
+        <v>6</v>
+      </c>
+      <c r="I9" s="1">
+        <v>6</v>
+      </c>
+      <c r="J9" s="1">
+        <v>6</v>
+      </c>
+      <c r="K9" s="1">
+        <v>6</v>
+      </c>
+      <c r="L9" s="1">
+        <v>6</v>
+      </c>
+      <c r="M9" s="1">
+        <v>6</v>
+      </c>
+      <c r="N9" s="1">
+        <v>6</v>
+      </c>
+      <c r="O9" s="1">
+        <v>6</v>
+      </c>
+      <c r="P9" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>7</v>
+      </c>
+      <c r="R9" s="1">
+        <v>7</v>
+      </c>
+      <c r="S9" s="1">
+        <v>7</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="U9" s="1">
+        <v>1</v>
+      </c>
+      <c r="U9" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>8</v>
-      </c>
-      <c r="B10" s="1">
-        <v>18</v>
-      </c>
-      <c r="C10" s="1">
-        <v>18</v>
-      </c>
-      <c r="D10" s="1">
-        <v>6</v>
-      </c>
-      <c r="E10" s="1">
-        <v>6</v>
-      </c>
-      <c r="F10" s="1">
-        <v>6</v>
-      </c>
-      <c r="G10" s="1">
-        <v>6</v>
-      </c>
-      <c r="H10" s="1">
-        <v>6</v>
-      </c>
-      <c r="I10" s="1">
-        <v>6</v>
-      </c>
-      <c r="J10" s="1">
-        <v>6</v>
-      </c>
-      <c r="K10" s="1">
-        <v>6</v>
-      </c>
-      <c r="L10" s="1">
-        <v>6</v>
-      </c>
-      <c r="M10" s="1">
-        <v>6</v>
-      </c>
-      <c r="N10" s="1">
-        <v>6</v>
-      </c>
-      <c r="O10" s="1">
-        <v>6</v>
-      </c>
-      <c r="P10" s="1">
-        <v>6</v>
-      </c>
-      <c r="Q10" s="1">
-        <v>18</v>
-      </c>
-      <c r="R10" s="1">
-        <v>18</v>
-      </c>
-      <c r="S10" s="1">
-        <v>18</v>
+        <v>7</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S10" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="U10" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="C11" s="1">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="D11" s="1">
         <v>6</v>
@@ -1238,7 +1256,7 @@
         <v>6</v>
       </c>
       <c r="M11" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="N11" s="1">
         <v>6</v>
@@ -1250,13 +1268,13 @@
         <v>6</v>
       </c>
       <c r="Q11" s="1">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="R11" s="1">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="S11" s="1">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="T11" s="1" t="s">
         <v>1</v>
@@ -1267,43 +1285,43 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
+        <v>9</v>
+      </c>
+      <c r="B12" s="1">
+        <v>21</v>
+      </c>
+      <c r="C12" s="1">
+        <v>21</v>
+      </c>
+      <c r="D12" s="1">
+        <v>6</v>
+      </c>
+      <c r="E12" s="1">
+        <v>6</v>
+      </c>
+      <c r="F12" s="1">
+        <v>6</v>
+      </c>
+      <c r="G12" s="1">
+        <v>6</v>
+      </c>
+      <c r="H12" s="1">
+        <v>6</v>
+      </c>
+      <c r="I12" s="1">
+        <v>6</v>
+      </c>
+      <c r="J12" s="1">
+        <v>6</v>
+      </c>
+      <c r="K12" s="1">
+        <v>6</v>
+      </c>
+      <c r="L12" s="1">
+        <v>6</v>
+      </c>
+      <c r="M12" s="1">
         <v>10</v>
-      </c>
-      <c r="B12" s="1">
-        <v>21</v>
-      </c>
-      <c r="C12" s="1">
-        <v>21</v>
-      </c>
-      <c r="D12" s="1">
-        <v>6</v>
-      </c>
-      <c r="E12" s="1">
-        <v>6</v>
-      </c>
-      <c r="F12" s="1">
-        <v>6</v>
-      </c>
-      <c r="G12" s="1">
-        <v>6</v>
-      </c>
-      <c r="H12" s="1">
-        <v>6</v>
-      </c>
-      <c r="I12" s="1">
-        <v>11</v>
-      </c>
-      <c r="J12" s="1">
-        <v>6</v>
-      </c>
-      <c r="K12" s="1">
-        <v>6</v>
-      </c>
-      <c r="L12" s="1">
-        <v>6</v>
-      </c>
-      <c r="M12" s="1">
-        <v>6</v>
       </c>
       <c r="N12" s="1">
         <v>6</v>
@@ -1332,37 +1350,37 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
+        <v>10</v>
+      </c>
+      <c r="B13" s="1">
+        <v>21</v>
+      </c>
+      <c r="C13" s="1">
+        <v>21</v>
+      </c>
+      <c r="D13" s="1">
+        <v>6</v>
+      </c>
+      <c r="E13" s="1">
+        <v>6</v>
+      </c>
+      <c r="F13" s="1">
+        <v>6</v>
+      </c>
+      <c r="G13" s="1">
+        <v>6</v>
+      </c>
+      <c r="H13" s="1">
+        <v>6</v>
+      </c>
+      <c r="I13" s="1">
         <v>11</v>
       </c>
-      <c r="B13" s="1">
-        <v>21</v>
-      </c>
-      <c r="C13" s="1">
-        <v>21</v>
-      </c>
-      <c r="D13" s="1">
-        <v>6</v>
-      </c>
-      <c r="E13" s="1">
-        <v>6</v>
-      </c>
-      <c r="F13" s="1">
-        <v>6</v>
-      </c>
-      <c r="G13" s="1">
-        <v>6</v>
-      </c>
-      <c r="H13" s="1">
-        <v>6</v>
-      </c>
-      <c r="I13" s="1">
-        <v>6</v>
-      </c>
       <c r="J13" s="1">
         <v>6</v>
       </c>
       <c r="K13" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L13" s="1">
         <v>6</v>
@@ -1397,38 +1415,38 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
+        <v>11</v>
+      </c>
+      <c r="B14" s="1">
+        <v>21</v>
+      </c>
+      <c r="C14" s="1">
+        <v>21</v>
+      </c>
+      <c r="D14" s="1">
+        <v>6</v>
+      </c>
+      <c r="E14" s="1">
+        <v>6</v>
+      </c>
+      <c r="F14" s="1">
+        <v>6</v>
+      </c>
+      <c r="G14" s="1">
+        <v>6</v>
+      </c>
+      <c r="H14" s="1">
+        <v>6</v>
+      </c>
+      <c r="I14" s="1">
+        <v>6</v>
+      </c>
+      <c r="J14" s="1">
+        <v>6</v>
+      </c>
+      <c r="K14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="1">
-        <v>21</v>
-      </c>
-      <c r="C14" s="1">
-        <v>21</v>
-      </c>
-      <c r="D14" s="1">
-        <v>6</v>
-      </c>
-      <c r="E14" s="1">
-        <v>6</v>
-      </c>
-      <c r="F14" s="1">
-        <v>6</v>
-      </c>
-      <c r="G14" s="1">
-        <v>6</v>
-      </c>
-      <c r="H14" s="1">
-        <v>6</v>
-      </c>
-      <c r="I14" s="1">
-        <v>6</v>
-      </c>
-      <c r="J14" s="1">
-        <v>6</v>
-      </c>
-      <c r="K14" s="1">
-        <v>6</v>
-      </c>
       <c r="L14" s="1">
         <v>6</v>
       </c>
@@ -1439,7 +1457,7 @@
         <v>6</v>
       </c>
       <c r="O14" s="1">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="P14" s="1">
         <v>6</v>
@@ -1462,7 +1480,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="1">
         <v>21</v>
@@ -1489,10 +1507,10 @@
         <v>6</v>
       </c>
       <c r="J15" s="1">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="K15" s="1">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="L15" s="1">
         <v>6</v>
@@ -1504,7 +1522,7 @@
         <v>6</v>
       </c>
       <c r="O15" s="1">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="P15" s="1">
         <v>6</v>
@@ -1527,37 +1545,37 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
+        <v>13</v>
+      </c>
+      <c r="B16" s="1">
+        <v>21</v>
+      </c>
+      <c r="C16" s="1">
+        <v>21</v>
+      </c>
+      <c r="D16" s="1">
+        <v>6</v>
+      </c>
+      <c r="E16" s="1">
+        <v>6</v>
+      </c>
+      <c r="F16" s="1">
+        <v>6</v>
+      </c>
+      <c r="G16" s="1">
+        <v>6</v>
+      </c>
+      <c r="H16" s="1">
+        <v>6</v>
+      </c>
+      <c r="I16" s="1">
+        <v>6</v>
+      </c>
+      <c r="J16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="1">
-        <v>21</v>
-      </c>
-      <c r="C16" s="1">
-        <v>21</v>
-      </c>
-      <c r="D16" s="1">
-        <v>6</v>
-      </c>
-      <c r="E16" s="1">
-        <v>6</v>
-      </c>
-      <c r="F16" s="1">
-        <v>6</v>
-      </c>
-      <c r="G16" s="1">
-        <v>6</v>
-      </c>
-      <c r="H16" s="1">
-        <v>6</v>
-      </c>
-      <c r="I16" s="1">
-        <v>6</v>
-      </c>
-      <c r="J16" s="1">
-        <v>6</v>
-      </c>
       <c r="K16" s="1">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="L16" s="1">
         <v>6</v>
@@ -1566,7 +1584,7 @@
         <v>6</v>
       </c>
       <c r="N16" s="1">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="O16" s="1">
         <v>6</v>
@@ -1592,46 +1610,46 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
+        <v>14</v>
+      </c>
+      <c r="B17" s="1">
+        <v>21</v>
+      </c>
+      <c r="C17" s="1">
+        <v>21</v>
+      </c>
+      <c r="D17" s="1">
+        <v>6</v>
+      </c>
+      <c r="E17" s="1">
+        <v>6</v>
+      </c>
+      <c r="F17" s="1">
+        <v>6</v>
+      </c>
+      <c r="G17" s="1">
+        <v>6</v>
+      </c>
+      <c r="H17" s="1">
+        <v>6</v>
+      </c>
+      <c r="I17" s="1">
+        <v>6</v>
+      </c>
+      <c r="J17" s="1">
+        <v>6</v>
+      </c>
+      <c r="K17" s="1">
+        <v>6</v>
+      </c>
+      <c r="L17" s="1">
+        <v>6</v>
+      </c>
+      <c r="M17" s="1">
+        <v>6</v>
+      </c>
+      <c r="N17" s="1">
         <v>15</v>
-      </c>
-      <c r="B17" s="1">
-        <v>21</v>
-      </c>
-      <c r="C17" s="1">
-        <v>21</v>
-      </c>
-      <c r="D17" s="1">
-        <v>6</v>
-      </c>
-      <c r="E17" s="1">
-        <v>6</v>
-      </c>
-      <c r="F17" s="1">
-        <v>16</v>
-      </c>
-      <c r="G17" s="1">
-        <v>6</v>
-      </c>
-      <c r="H17" s="1">
-        <v>6</v>
-      </c>
-      <c r="I17" s="1">
-        <v>6</v>
-      </c>
-      <c r="J17" s="1">
-        <v>6</v>
-      </c>
-      <c r="K17" s="1">
-        <v>6</v>
-      </c>
-      <c r="L17" s="1">
-        <v>6</v>
-      </c>
-      <c r="M17" s="1">
-        <v>6</v>
-      </c>
-      <c r="N17" s="1">
-        <v>6</v>
       </c>
       <c r="O17" s="1">
         <v>6</v>
@@ -1657,23 +1675,23 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
+        <v>15</v>
+      </c>
+      <c r="B18" s="1">
+        <v>21</v>
+      </c>
+      <c r="C18" s="1">
+        <v>21</v>
+      </c>
+      <c r="D18" s="1">
+        <v>6</v>
+      </c>
+      <c r="E18" s="1">
+        <v>6</v>
+      </c>
+      <c r="F18" s="1">
         <v>16</v>
       </c>
-      <c r="B18" s="1">
-        <v>18</v>
-      </c>
-      <c r="C18" s="1">
-        <v>18</v>
-      </c>
-      <c r="D18" s="1">
-        <v>6</v>
-      </c>
-      <c r="E18" s="1">
-        <v>6</v>
-      </c>
-      <c r="F18" s="1">
-        <v>6</v>
-      </c>
       <c r="G18" s="1">
         <v>6</v>
       </c>
@@ -1705,13 +1723,13 @@
         <v>6</v>
       </c>
       <c r="Q18" s="1">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="R18" s="1">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="S18" s="1">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="T18" s="1" t="s">
         <v>1</v>
@@ -1722,72 +1740,72 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>17</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="N19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="O19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="S19" s="1" t="s">
-        <v>1</v>
+        <v>16</v>
+      </c>
+      <c r="B19" s="1">
+        <v>18</v>
+      </c>
+      <c r="C19" s="1">
+        <v>18</v>
+      </c>
+      <c r="D19" s="1">
+        <v>6</v>
+      </c>
+      <c r="E19" s="1">
+        <v>6</v>
+      </c>
+      <c r="F19" s="1">
+        <v>6</v>
+      </c>
+      <c r="G19" s="1">
+        <v>6</v>
+      </c>
+      <c r="H19" s="1">
+        <v>6</v>
+      </c>
+      <c r="I19" s="1">
+        <v>6</v>
+      </c>
+      <c r="J19" s="1">
+        <v>6</v>
+      </c>
+      <c r="K19" s="1">
+        <v>6</v>
+      </c>
+      <c r="L19" s="1">
+        <v>6</v>
+      </c>
+      <c r="M19" s="1">
+        <v>6</v>
+      </c>
+      <c r="N19" s="1">
+        <v>6</v>
+      </c>
+      <c r="O19" s="1">
+        <v>6</v>
+      </c>
+      <c r="P19" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q19" s="1">
+        <v>18</v>
+      </c>
+      <c r="R19" s="1">
+        <v>18</v>
+      </c>
+      <c r="S19" s="1">
+        <v>18</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="U19" s="1">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="U19" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>1</v>
@@ -1844,15 +1862,15 @@
         <v>1</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="U20" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>1</v>
@@ -1909,15 +1927,15 @@
         <v>1</v>
       </c>
       <c r="T21" s="1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="U21" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>1</v>
@@ -1974,7 +1992,7 @@
         <v>1</v>
       </c>
       <c r="T22" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="U22" s="1">
         <v>0</v>
@@ -1982,7 +2000,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>1</v>
@@ -2039,86 +2057,86 @@
         <v>1</v>
       </c>
       <c r="T23" s="1" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="U23" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>22</v>
-      </c>
-      <c r="B24" s="1">
-        <v>18</v>
-      </c>
-      <c r="C24" s="1">
-        <v>18</v>
-      </c>
-      <c r="D24" s="1">
-        <v>6</v>
-      </c>
-      <c r="E24" s="1">
-        <v>6</v>
-      </c>
-      <c r="F24" s="1">
-        <v>6</v>
-      </c>
-      <c r="G24" s="1">
-        <v>6</v>
-      </c>
-      <c r="H24" s="1">
-        <v>6</v>
-      </c>
-      <c r="I24" s="1">
-        <v>6</v>
-      </c>
-      <c r="J24" s="1">
-        <v>6</v>
-      </c>
-      <c r="K24" s="1">
-        <v>6</v>
-      </c>
-      <c r="L24" s="1">
-        <v>6</v>
-      </c>
-      <c r="M24" s="1">
-        <v>6</v>
-      </c>
-      <c r="N24" s="1">
-        <v>6</v>
-      </c>
-      <c r="O24" s="1">
-        <v>6</v>
-      </c>
-      <c r="P24" s="1">
-        <v>6</v>
-      </c>
-      <c r="Q24" s="1">
-        <v>18</v>
-      </c>
-      <c r="R24" s="1">
-        <v>18</v>
-      </c>
-      <c r="S24" s="1">
-        <v>18</v>
+        <v>21</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S24" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="T24" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U24" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="U24" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B25" s="1">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C25" s="1">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D25" s="1">
         <v>6</v>
@@ -2127,7 +2145,7 @@
         <v>6</v>
       </c>
       <c r="F25" s="1">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="G25" s="1">
         <v>6</v>
@@ -2160,13 +2178,13 @@
         <v>6</v>
       </c>
       <c r="Q25" s="1">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="R25" s="1">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="S25" s="1">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="T25" s="1" t="s">
         <v>1</v>
@@ -2177,28 +2195,28 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
+        <v>23</v>
+      </c>
+      <c r="B26" s="1">
+        <v>33</v>
+      </c>
+      <c r="C26" s="1">
+        <v>33</v>
+      </c>
+      <c r="D26" s="1">
+        <v>6</v>
+      </c>
+      <c r="E26" s="1">
+        <v>6</v>
+      </c>
+      <c r="F26" s="1">
         <v>24</v>
       </c>
-      <c r="B26" s="1">
-        <v>33</v>
-      </c>
-      <c r="C26" s="1">
-        <v>33</v>
-      </c>
-      <c r="D26" s="1">
-        <v>6</v>
-      </c>
-      <c r="E26" s="1">
-        <v>6</v>
-      </c>
-      <c r="F26" s="1">
-        <v>6</v>
-      </c>
       <c r="G26" s="1">
         <v>6</v>
       </c>
       <c r="H26" s="1">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="I26" s="1">
         <v>6</v>
@@ -2242,31 +2260,31 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
+        <v>24</v>
+      </c>
+      <c r="B27" s="1">
+        <v>33</v>
+      </c>
+      <c r="C27" s="1">
+        <v>33</v>
+      </c>
+      <c r="D27" s="1">
+        <v>6</v>
+      </c>
+      <c r="E27" s="1">
+        <v>6</v>
+      </c>
+      <c r="F27" s="1">
+        <v>6</v>
+      </c>
+      <c r="G27" s="1">
+        <v>6</v>
+      </c>
+      <c r="H27" s="1">
         <v>25</v>
       </c>
-      <c r="B27" s="1">
-        <v>33</v>
-      </c>
-      <c r="C27" s="1">
-        <v>33</v>
-      </c>
-      <c r="D27" s="1">
-        <v>6</v>
-      </c>
-      <c r="E27" s="1">
-        <v>6</v>
-      </c>
-      <c r="F27" s="1">
-        <v>6</v>
-      </c>
-      <c r="G27" s="1">
-        <v>6</v>
-      </c>
-      <c r="H27" s="1">
-        <v>6</v>
-      </c>
       <c r="I27" s="1">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="J27" s="1">
         <v>6</v>
@@ -2307,37 +2325,37 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
+        <v>25</v>
+      </c>
+      <c r="B28" s="1">
+        <v>33</v>
+      </c>
+      <c r="C28" s="1">
+        <v>33</v>
+      </c>
+      <c r="D28" s="1">
+        <v>6</v>
+      </c>
+      <c r="E28" s="1">
+        <v>6</v>
+      </c>
+      <c r="F28" s="1">
+        <v>6</v>
+      </c>
+      <c r="G28" s="1">
+        <v>6</v>
+      </c>
+      <c r="H28" s="1">
+        <v>6</v>
+      </c>
+      <c r="I28" s="1">
         <v>26</v>
       </c>
-      <c r="B28" s="1">
-        <v>33</v>
-      </c>
-      <c r="C28" s="1">
-        <v>33</v>
-      </c>
-      <c r="D28" s="1">
-        <v>6</v>
-      </c>
-      <c r="E28" s="1">
-        <v>6</v>
-      </c>
-      <c r="F28" s="1">
-        <v>6</v>
-      </c>
-      <c r="G28" s="1">
-        <v>6</v>
-      </c>
-      <c r="H28" s="1">
-        <v>6</v>
-      </c>
-      <c r="I28" s="1">
-        <v>6</v>
-      </c>
       <c r="J28" s="1">
         <v>6</v>
       </c>
       <c r="K28" s="1">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="L28" s="1">
         <v>6</v>
@@ -2372,38 +2390,38 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
+        <v>26</v>
+      </c>
+      <c r="B29" s="1">
+        <v>33</v>
+      </c>
+      <c r="C29" s="1">
+        <v>33</v>
+      </c>
+      <c r="D29" s="1">
+        <v>6</v>
+      </c>
+      <c r="E29" s="1">
+        <v>6</v>
+      </c>
+      <c r="F29" s="1">
+        <v>6</v>
+      </c>
+      <c r="G29" s="1">
+        <v>6</v>
+      </c>
+      <c r="H29" s="1">
+        <v>6</v>
+      </c>
+      <c r="I29" s="1">
+        <v>6</v>
+      </c>
+      <c r="J29" s="1">
+        <v>6</v>
+      </c>
+      <c r="K29" s="1">
         <v>27</v>
       </c>
-      <c r="B29" s="1">
-        <v>18</v>
-      </c>
-      <c r="C29" s="1">
-        <v>18</v>
-      </c>
-      <c r="D29" s="1">
-        <v>6</v>
-      </c>
-      <c r="E29" s="1">
-        <v>6</v>
-      </c>
-      <c r="F29" s="1">
-        <v>6</v>
-      </c>
-      <c r="G29" s="1">
-        <v>6</v>
-      </c>
-      <c r="H29" s="1">
-        <v>6</v>
-      </c>
-      <c r="I29" s="1">
-        <v>6</v>
-      </c>
-      <c r="J29" s="1">
-        <v>6</v>
-      </c>
-      <c r="K29" s="1">
-        <v>6</v>
-      </c>
       <c r="L29" s="1">
         <v>6</v>
       </c>
@@ -2420,13 +2438,13 @@
         <v>6</v>
       </c>
       <c r="Q29" s="1">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="R29" s="1">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="S29" s="1">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="T29" s="1" t="s">
         <v>1</v>
@@ -2437,19 +2455,19 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B30" s="1">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="C30" s="1">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="D30" s="1">
         <v>6</v>
       </c>
       <c r="E30" s="1">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="F30" s="1">
         <v>6</v>
@@ -2485,13 +2503,13 @@
         <v>6</v>
       </c>
       <c r="Q30" s="1">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="R30" s="1">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="S30" s="1">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="T30" s="1" t="s">
         <v>1</v>
@@ -2502,20 +2520,20 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
+        <v>28</v>
+      </c>
+      <c r="B31" s="1">
+        <v>21</v>
+      </c>
+      <c r="C31" s="1">
+        <v>21</v>
+      </c>
+      <c r="D31" s="1">
+        <v>6</v>
+      </c>
+      <c r="E31" s="1">
         <v>29</v>
       </c>
-      <c r="B31" s="1">
-        <v>18</v>
-      </c>
-      <c r="C31" s="1">
-        <v>18</v>
-      </c>
-      <c r="D31" s="1">
-        <v>6</v>
-      </c>
-      <c r="E31" s="1">
-        <v>6</v>
-      </c>
       <c r="F31" s="1">
         <v>6</v>
       </c>
@@ -2550,13 +2568,13 @@
         <v>6</v>
       </c>
       <c r="Q31" s="1">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="R31" s="1">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="S31" s="1">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="T31" s="1" t="s">
         <v>1</v>
@@ -2567,13 +2585,13 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B32" s="1">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C32" s="1">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="D32" s="1">
         <v>6</v>
@@ -2582,7 +2600,7 @@
         <v>6</v>
       </c>
       <c r="F32" s="1">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="G32" s="1">
         <v>6</v>
@@ -2615,13 +2633,13 @@
         <v>6</v>
       </c>
       <c r="Q32" s="1">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="R32" s="1">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="S32" s="1">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="T32" s="1" t="s">
         <v>1</v>
@@ -2632,25 +2650,25 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
+        <v>30</v>
+      </c>
+      <c r="B33" s="1">
+        <v>33</v>
+      </c>
+      <c r="C33" s="1">
+        <v>33</v>
+      </c>
+      <c r="D33" s="1">
+        <v>6</v>
+      </c>
+      <c r="E33" s="1">
+        <v>6</v>
+      </c>
+      <c r="F33" s="1">
         <v>31</v>
       </c>
-      <c r="B33" s="1">
-        <v>33</v>
-      </c>
-      <c r="C33" s="1">
-        <v>33</v>
-      </c>
-      <c r="D33" s="1">
-        <v>6</v>
-      </c>
-      <c r="E33" s="1">
-        <v>6</v>
-      </c>
-      <c r="F33" s="1">
-        <v>6</v>
-      </c>
       <c r="G33" s="1">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="H33" s="1">
         <v>6</v>
@@ -2697,26 +2715,26 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
+        <v>31</v>
+      </c>
+      <c r="B34" s="1">
+        <v>33</v>
+      </c>
+      <c r="C34" s="1">
+        <v>33</v>
+      </c>
+      <c r="D34" s="1">
+        <v>6</v>
+      </c>
+      <c r="E34" s="1">
+        <v>6</v>
+      </c>
+      <c r="F34" s="1">
+        <v>6</v>
+      </c>
+      <c r="G34" s="1">
         <v>32</v>
       </c>
-      <c r="B34" s="1">
-        <v>18</v>
-      </c>
-      <c r="C34" s="1">
-        <v>18</v>
-      </c>
-      <c r="D34" s="1">
-        <v>6</v>
-      </c>
-      <c r="E34" s="1">
-        <v>6</v>
-      </c>
-      <c r="F34" s="1">
-        <v>6</v>
-      </c>
-      <c r="G34" s="1">
-        <v>6</v>
-      </c>
       <c r="H34" s="1">
         <v>6</v>
       </c>
@@ -2745,13 +2763,13 @@
         <v>6</v>
       </c>
       <c r="Q34" s="1">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="R34" s="1">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="S34" s="1">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="T34" s="1" t="s">
         <v>1</v>
@@ -2762,66 +2780,463 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>33</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="M35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="S35" s="1" t="s">
-        <v>1</v>
+        <v>32</v>
+      </c>
+      <c r="B35" s="1">
+        <v>39</v>
+      </c>
+      <c r="C35" s="1">
+        <v>39</v>
+      </c>
+      <c r="D35" s="1">
+        <v>6</v>
+      </c>
+      <c r="E35" s="1">
+        <v>6</v>
+      </c>
+      <c r="F35" s="1">
+        <v>6</v>
+      </c>
+      <c r="G35" s="1">
+        <v>6</v>
+      </c>
+      <c r="H35" s="1">
+        <v>6</v>
+      </c>
+      <c r="I35" s="1">
+        <v>6</v>
+      </c>
+      <c r="J35" s="1">
+        <v>6</v>
+      </c>
+      <c r="K35" s="1">
+        <v>6</v>
+      </c>
+      <c r="L35" s="1">
+        <v>6</v>
+      </c>
+      <c r="M35" s="1">
+        <v>6</v>
+      </c>
+      <c r="N35" s="1">
+        <v>6</v>
+      </c>
+      <c r="O35" s="1">
+        <v>6</v>
+      </c>
+      <c r="P35" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q35" s="1">
+        <v>39</v>
+      </c>
+      <c r="R35" s="1">
+        <v>39</v>
+      </c>
+      <c r="S35" s="1">
+        <v>39</v>
       </c>
       <c r="T35" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="U35" s="1">
+        <v>1</v>
+      </c>
+      <c r="U35" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>33</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T36" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="U36" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>34</v>
+      </c>
+      <c r="T37" s="1"/>
+      <c r="U37" s="1"/>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>35</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T38" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="U38" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>36</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T39" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U39" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>37</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T40" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="U40" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>38</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S41" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T41" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="U41" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>39</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T42" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="U42" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>